<commit_message>
Indicadores: con TEMPORALES y  ALCON Y  HISTÓRICO listos
</commit_message>
<xml_diff>
--- a/datos/salida/Indicadores_operacion_nuevo.xlsx
+++ b/datos/salida/Indicadores_operacion_nuevo.xlsx
@@ -55,12 +55,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -426,9 +428,475 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A81:E230"/>
+  <dimension ref="A4:E503"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Area</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>TOTAL CUENTAS TEMPORALES CON SALDO</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>CUENTAS TEMPORALES FUERA DE POLITICA</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>EVC SERVICIOS ESTRATEGICOS NEGOCIO LRU</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="C5" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="D5" s="2">
+        <f>IFERROR(C5/B5,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>EVC SERVICIOS PARA EL NEGOCIO SUFI</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="C6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" s="2">
+        <f>IFERROR(C6/B6,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>GCIA ATENCION AL CLIENTE</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" s="2">
+        <f>IFERROR(C7/B7,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>GCIA AUTOSERVICIOS Y EFECTIVO</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="C8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D8" s="2">
+        <f>IFERROR(C8/B8,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>GCIA CONTABLE Y TRIBUTARIA NEQUI</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="n">
+        <v>26</v>
+      </c>
+      <c r="C9" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="D9" s="2">
+        <f>IFERROR(C9/B9,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>GCIA DE REQUERIMIENTOS LEGALES E INSTITU</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" s="2">
+        <f>IFERROR(C10/B10,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>GCIA DE SERV REPORTERIA LEGAL Y TRIBUT</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D11" s="2">
+        <f>IFERROR(C11/B11,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>GCIA LIMITES DESEMBOLSOS Y GARANTIAS</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D12" s="2">
+        <f>IFERROR(C12/B12,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>GCIA OP NEGOCIO INMOBILIARIO Y FACTORING</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="C13" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="D13" s="2">
+        <f>IFERROR(C13/B13,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>GCIA OPERACION DEPOSITOS PARA CLIENTES</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="C14" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="D14" s="2">
+        <f>IFERROR(C14/B14,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>GCIA OPERACION MEDIOS Y ACEPTACION PAGOS</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="n">
+        <v>81</v>
+      </c>
+      <c r="C15" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="D15" s="2">
+        <f>IFERROR(C15/B15,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>GCIA OPERACIONES SEGUROS Y NUEVOS FLUJOS</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C16" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D16" s="2">
+        <f>IFERROR(C16/B16,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>GCIA SERV FINANCIEROS MERCADO CAPITALES</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="C17" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D17" s="2">
+        <f>IFERROR(C17/B17,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>GCIA SERVICIOS CONTABLES ADMINISTRATIVOS</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="C18" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="D18" s="2">
+        <f>IFERROR(C18/B18,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>GCIA SERVICIOS DE NOMINA A EMPLEADOS</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="C19" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D19" s="2">
+        <f>IFERROR(C19/B19,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>GCIA SERVICIOS FINANCIEROS CORPORATIVOS</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C20" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D20" s="2">
+        <f>IFERROR(C20/B20,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>GCIA SERVICIOS GESTION DEL FRAUDE</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="C21" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D21" s="2">
+        <f>IFERROR(C21/B21,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>GCIA SERVICIOS INVERSIONES Y TESORERIA</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C22" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D22" s="2">
+        <f>IFERROR(C22/B22,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>GERENCIA DE SERVICIOS DE COBRANZA Y BRP</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="C23" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="D23" s="2">
+        <f>IFERROR(C23/B23,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>GERENCIA OPERACION CASH MANAGEMENT</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C24" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D24" s="2">
+        <f>IFERROR(C24/B24,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>GERENCIA OPERACION DE FINANCIACION</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="C25" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D25" s="2">
+        <f>IFERROR(C25/B25,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>LDC PRODUCTO VIDA Y SALUD</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C26" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D26" s="2">
+        <f>IFERROR(C26/B26,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Total general</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="n">
+        <v>187</v>
+      </c>
+      <c r="C27" s="4" t="n">
+        <v>49</v>
+      </c>
+      <c r="D27" s="2">
+        <f>IFERROR(C27/B27,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28"/>
+    <row r="29"/>
+    <row r="30"/>
+    <row r="31"/>
+    <row r="32"/>
+    <row r="33"/>
+    <row r="34"/>
+    <row r="35"/>
+    <row r="36"/>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39"/>
+    <row r="40"/>
+    <row r="41"/>
+    <row r="42"/>
+    <row r="43"/>
+    <row r="44"/>
+    <row r="45"/>
+    <row r="46"/>
+    <row r="47"/>
+    <row r="48"/>
+    <row r="49"/>
+    <row r="50"/>
+    <row r="51"/>
+    <row r="52"/>
+    <row r="53"/>
+    <row r="54"/>
+    <row r="55"/>
+    <row r="56"/>
+    <row r="57"/>
+    <row r="58"/>
+    <row r="59"/>
+    <row r="60"/>
+    <row r="61"/>
+    <row r="62"/>
+    <row r="63"/>
+    <row r="64"/>
+    <row r="65"/>
+    <row r="66"/>
+    <row r="67"/>
+    <row r="68"/>
+    <row r="69"/>
+    <row r="70"/>
+    <row r="71"/>
+    <row r="72"/>
+    <row r="73"/>
+    <row r="74"/>
+    <row r="75"/>
+    <row r="76"/>
+    <row r="77"/>
+    <row r="78"/>
+    <row r="79"/>
+    <row r="80"/>
     <row r="81">
       <c r="A81" s="1" t="inlineStr">
         <is>
@@ -1140,6 +1608,68 @@
         <v>0.006652526031623585</v>
       </c>
     </row>
+    <row r="118"/>
+    <row r="119"/>
+    <row r="120"/>
+    <row r="121"/>
+    <row r="122"/>
+    <row r="123"/>
+    <row r="124"/>
+    <row r="125"/>
+    <row r="126"/>
+    <row r="127"/>
+    <row r="128"/>
+    <row r="129"/>
+    <row r="130"/>
+    <row r="131"/>
+    <row r="132"/>
+    <row r="133"/>
+    <row r="134"/>
+    <row r="135"/>
+    <row r="136"/>
+    <row r="137"/>
+    <row r="138"/>
+    <row r="139"/>
+    <row r="140"/>
+    <row r="141"/>
+    <row r="142"/>
+    <row r="143"/>
+    <row r="144"/>
+    <row r="145"/>
+    <row r="146"/>
+    <row r="147"/>
+    <row r="148"/>
+    <row r="149"/>
+    <row r="150"/>
+    <row r="151"/>
+    <row r="152"/>
+    <row r="153"/>
+    <row r="154"/>
+    <row r="155"/>
+    <row r="156"/>
+    <row r="157"/>
+    <row r="158"/>
+    <row r="159"/>
+    <row r="160"/>
+    <row r="161"/>
+    <row r="162"/>
+    <row r="163"/>
+    <row r="164"/>
+    <row r="165"/>
+    <row r="166"/>
+    <row r="167"/>
+    <row r="168"/>
+    <row r="169"/>
+    <row r="170"/>
+    <row r="171"/>
+    <row r="172"/>
+    <row r="173"/>
+    <row r="174"/>
+    <row r="175"/>
+    <row r="176"/>
+    <row r="177"/>
+    <row r="178"/>
+    <row r="179"/>
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
@@ -2128,9 +2658,6 @@
           <t>*El indicador mide el incumplimiento en función de los días calendario del mes. Cada día de atraso tiene el mismo peso, independientemente de la fecha objetivo.</t>
         </is>
       </c>
-      <c r="B229" t="inlineStr"/>
-      <c r="C229" t="inlineStr"/>
-      <c r="D229" t="inlineStr"/>
     </row>
     <row r="230">
       <c r="C230" t="inlineStr">
@@ -2143,6 +2670,279 @@
         <v/>
       </c>
     </row>
+    <row r="231"/>
+    <row r="232"/>
+    <row r="233"/>
+    <row r="234"/>
+    <row r="235"/>
+    <row r="236"/>
+    <row r="237"/>
+    <row r="238"/>
+    <row r="239"/>
+    <row r="240"/>
+    <row r="241"/>
+    <row r="242"/>
+    <row r="243"/>
+    <row r="244"/>
+    <row r="245"/>
+    <row r="246"/>
+    <row r="247"/>
+    <row r="248"/>
+    <row r="249"/>
+    <row r="250"/>
+    <row r="251"/>
+    <row r="252"/>
+    <row r="253"/>
+    <row r="254"/>
+    <row r="255"/>
+    <row r="256"/>
+    <row r="257"/>
+    <row r="258"/>
+    <row r="259"/>
+    <row r="260"/>
+    <row r="261"/>
+    <row r="262"/>
+    <row r="263"/>
+    <row r="264"/>
+    <row r="265"/>
+    <row r="266"/>
+    <row r="267"/>
+    <row r="268"/>
+    <row r="269"/>
+    <row r="270"/>
+    <row r="271"/>
+    <row r="272"/>
+    <row r="273"/>
+    <row r="274"/>
+    <row r="275"/>
+    <row r="276"/>
+    <row r="277"/>
+    <row r="278"/>
+    <row r="279"/>
+    <row r="280"/>
+    <row r="281"/>
+    <row r="282"/>
+    <row r="283"/>
+    <row r="284"/>
+    <row r="285"/>
+    <row r="286"/>
+    <row r="287"/>
+    <row r="288"/>
+    <row r="289"/>
+    <row r="290"/>
+    <row r="291"/>
+    <row r="292"/>
+    <row r="293"/>
+    <row r="294"/>
+    <row r="295"/>
+    <row r="296"/>
+    <row r="297"/>
+    <row r="298"/>
+    <row r="299"/>
+    <row r="300"/>
+    <row r="301"/>
+    <row r="302"/>
+    <row r="303"/>
+    <row r="304"/>
+    <row r="305"/>
+    <row r="306"/>
+    <row r="307"/>
+    <row r="308"/>
+    <row r="309"/>
+    <row r="310"/>
+    <row r="311"/>
+    <row r="312"/>
+    <row r="313"/>
+    <row r="314"/>
+    <row r="315"/>
+    <row r="316"/>
+    <row r="317"/>
+    <row r="318"/>
+    <row r="319"/>
+    <row r="320"/>
+    <row r="321"/>
+    <row r="322"/>
+    <row r="323"/>
+    <row r="324"/>
+    <row r="325"/>
+    <row r="326"/>
+    <row r="327"/>
+    <row r="328"/>
+    <row r="329"/>
+    <row r="330"/>
+    <row r="331"/>
+    <row r="332"/>
+    <row r="333"/>
+    <row r="334"/>
+    <row r="335"/>
+    <row r="336"/>
+    <row r="337"/>
+    <row r="338"/>
+    <row r="339"/>
+    <row r="340"/>
+    <row r="341"/>
+    <row r="342"/>
+    <row r="343"/>
+    <row r="344"/>
+    <row r="345"/>
+    <row r="346"/>
+    <row r="347"/>
+    <row r="348"/>
+    <row r="349"/>
+    <row r="350"/>
+    <row r="351"/>
+    <row r="352"/>
+    <row r="353"/>
+    <row r="354"/>
+    <row r="355"/>
+    <row r="356"/>
+    <row r="357"/>
+    <row r="358"/>
+    <row r="359"/>
+    <row r="360"/>
+    <row r="361"/>
+    <row r="362"/>
+    <row r="363"/>
+    <row r="364"/>
+    <row r="365"/>
+    <row r="366"/>
+    <row r="367"/>
+    <row r="368"/>
+    <row r="369"/>
+    <row r="370"/>
+    <row r="371"/>
+    <row r="372"/>
+    <row r="373"/>
+    <row r="374"/>
+    <row r="375"/>
+    <row r="376"/>
+    <row r="377"/>
+    <row r="378"/>
+    <row r="379"/>
+    <row r="380"/>
+    <row r="381"/>
+    <row r="382"/>
+    <row r="383"/>
+    <row r="384"/>
+    <row r="385"/>
+    <row r="386"/>
+    <row r="387"/>
+    <row r="388"/>
+    <row r="389"/>
+    <row r="390"/>
+    <row r="391"/>
+    <row r="392"/>
+    <row r="393"/>
+    <row r="394"/>
+    <row r="395"/>
+    <row r="396"/>
+    <row r="397"/>
+    <row r="398"/>
+    <row r="399"/>
+    <row r="400"/>
+    <row r="401"/>
+    <row r="402"/>
+    <row r="403"/>
+    <row r="404"/>
+    <row r="405"/>
+    <row r="406"/>
+    <row r="407"/>
+    <row r="408"/>
+    <row r="409"/>
+    <row r="410"/>
+    <row r="411"/>
+    <row r="412"/>
+    <row r="413"/>
+    <row r="414"/>
+    <row r="415"/>
+    <row r="416"/>
+    <row r="417"/>
+    <row r="418"/>
+    <row r="419"/>
+    <row r="420"/>
+    <row r="421"/>
+    <row r="422"/>
+    <row r="423"/>
+    <row r="424"/>
+    <row r="425"/>
+    <row r="426"/>
+    <row r="427"/>
+    <row r="428"/>
+    <row r="429"/>
+    <row r="430"/>
+    <row r="431"/>
+    <row r="432"/>
+    <row r="433"/>
+    <row r="434"/>
+    <row r="435"/>
+    <row r="436"/>
+    <row r="437"/>
+    <row r="438"/>
+    <row r="439"/>
+    <row r="440"/>
+    <row r="441"/>
+    <row r="442"/>
+    <row r="443"/>
+    <row r="444"/>
+    <row r="445"/>
+    <row r="446"/>
+    <row r="447"/>
+    <row r="448"/>
+    <row r="449"/>
+    <row r="450"/>
+    <row r="451"/>
+    <row r="452"/>
+    <row r="453"/>
+    <row r="454"/>
+    <row r="455"/>
+    <row r="456"/>
+    <row r="457"/>
+    <row r="458"/>
+    <row r="459"/>
+    <row r="460"/>
+    <row r="461"/>
+    <row r="462"/>
+    <row r="463"/>
+    <row r="464"/>
+    <row r="465"/>
+    <row r="466"/>
+    <row r="467"/>
+    <row r="468"/>
+    <row r="469"/>
+    <row r="470"/>
+    <row r="471"/>
+    <row r="472"/>
+    <row r="473"/>
+    <row r="474"/>
+    <row r="475"/>
+    <row r="476"/>
+    <row r="477"/>
+    <row r="478"/>
+    <row r="479"/>
+    <row r="480"/>
+    <row r="481"/>
+    <row r="482"/>
+    <row r="483"/>
+    <row r="484"/>
+    <row r="485"/>
+    <row r="486"/>
+    <row r="487"/>
+    <row r="488"/>
+    <row r="489"/>
+    <row r="490"/>
+    <row r="491"/>
+    <row r="492"/>
+    <row r="493"/>
+    <row r="494"/>
+    <row r="495"/>
+    <row r="496"/>
+    <row r="497"/>
+    <row r="498"/>
+    <row r="499"/>
+    <row r="500"/>
+    <row r="501"/>
+    <row r="502"/>
+    <row r="503"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
TD sabana, traslado a indicadores y copia local de Temporales
</commit_message>
<xml_diff>
--- a/datos/salida/Indicadores_operacion_nuevo.xlsx
+++ b/datos/salida/Indicadores_operacion_nuevo.xlsx
@@ -16,7 +16,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.0%"/>
+  </numFmts>
   <fonts count="2">
     <font>
       <name val="Calibri"/>
@@ -55,7 +57,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
@@ -63,6 +65,7 @@
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -428,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A4:E503"/>
+  <dimension ref="A4:G503"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="4">
@@ -452,6 +455,21 @@
           <t>%</t>
         </is>
       </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>TOTAL PARTIDAS</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>PARTIDAS FUERA DE POLITICA</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -469,6 +487,16 @@
         <f>IFERROR(C5/B5,0)</f>
         <v/>
       </c>
+      <c r="E5" s="4" t="n">
+        <v>448</v>
+      </c>
+      <c r="F5" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="G5" s="5">
+        <f>IFERROR(F5/E5,0)</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -486,6 +514,16 @@
         <f>IFERROR(C6/B6,0)</f>
         <v/>
       </c>
+      <c r="E6" s="4" t="n">
+        <v>5504</v>
+      </c>
+      <c r="F6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" s="5">
+        <f>IFERROR(F6/E6,0)</f>
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -503,6 +541,16 @@
         <f>IFERROR(C7/B7,0)</f>
         <v/>
       </c>
+      <c r="E7" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="F7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" s="5">
+        <f>IFERROR(F7/E7,0)</f>
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -520,6 +568,16 @@
         <f>IFERROR(C8/B8,0)</f>
         <v/>
       </c>
+      <c r="E8" s="4" t="n">
+        <v>3322</v>
+      </c>
+      <c r="F8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" s="5">
+        <f>IFERROR(F8/E8,0)</f>
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -537,6 +595,16 @@
         <f>IFERROR(C9/B9,0)</f>
         <v/>
       </c>
+      <c r="E9" s="4" t="n">
+        <v>29529</v>
+      </c>
+      <c r="F9" s="4" t="n">
+        <v>161</v>
+      </c>
+      <c r="G9" s="5">
+        <f>IFERROR(F9/E9,0)</f>
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -554,6 +622,16 @@
         <f>IFERROR(C10/B10,0)</f>
         <v/>
       </c>
+      <c r="E10" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="F10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" s="5">
+        <f>IFERROR(F10/E10,0)</f>
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -571,6 +649,16 @@
         <f>IFERROR(C11/B11,0)</f>
         <v/>
       </c>
+      <c r="E11" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="F11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" s="5">
+        <f>IFERROR(F11/E11,0)</f>
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -588,6 +676,16 @@
         <f>IFERROR(C12/B12,0)</f>
         <v/>
       </c>
+      <c r="E12" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" s="5">
+        <f>IFERROR(F12/E12,0)</f>
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -605,6 +703,16 @@
         <f>IFERROR(C13/B13,0)</f>
         <v/>
       </c>
+      <c r="E13" s="4" t="n">
+        <v>2251</v>
+      </c>
+      <c r="F13" s="4" t="n">
+        <v>46</v>
+      </c>
+      <c r="G13" s="5">
+        <f>IFERROR(F13/E13,0)</f>
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -622,6 +730,16 @@
         <f>IFERROR(C14/B14,0)</f>
         <v/>
       </c>
+      <c r="E14" s="4" t="n">
+        <v>1014</v>
+      </c>
+      <c r="F14" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="G14" s="5">
+        <f>IFERROR(F14/E14,0)</f>
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -639,6 +757,16 @@
         <f>IFERROR(C15/B15,0)</f>
         <v/>
       </c>
+      <c r="E15" s="4" t="n">
+        <v>357459</v>
+      </c>
+      <c r="F15" s="4" t="n">
+        <v>4040</v>
+      </c>
+      <c r="G15" s="5">
+        <f>IFERROR(F15/E15,0)</f>
+        <v/>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -656,6 +784,16 @@
         <f>IFERROR(C16/B16,0)</f>
         <v/>
       </c>
+      <c r="E16" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F16" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G16" s="5">
+        <f>IFERROR(F16/E16,0)</f>
+        <v/>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -673,6 +811,16 @@
         <f>IFERROR(C17/B17,0)</f>
         <v/>
       </c>
+      <c r="E17" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="F17" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G17" s="5">
+        <f>IFERROR(F17/E17,0)</f>
+        <v/>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -690,6 +838,16 @@
         <f>IFERROR(C18/B18,0)</f>
         <v/>
       </c>
+      <c r="E18" s="4" t="n">
+        <v>473</v>
+      </c>
+      <c r="F18" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="G18" s="5">
+        <f>IFERROR(F18/E18,0)</f>
+        <v/>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -707,6 +865,16 @@
         <f>IFERROR(C19/B19,0)</f>
         <v/>
       </c>
+      <c r="E19" s="4" t="n">
+        <v>60</v>
+      </c>
+      <c r="F19" s="4" t="n">
+        <v>29</v>
+      </c>
+      <c r="G19" s="5">
+        <f>IFERROR(F19/E19,0)</f>
+        <v/>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -724,6 +892,16 @@
         <f>IFERROR(C20/B20,0)</f>
         <v/>
       </c>
+      <c r="E20" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F20" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G20" s="5">
+        <f>IFERROR(F20/E20,0)</f>
+        <v/>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -741,6 +919,16 @@
         <f>IFERROR(C21/B21,0)</f>
         <v/>
       </c>
+      <c r="E21" s="4" t="n">
+        <v>15908</v>
+      </c>
+      <c r="F21" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="G21" s="5">
+        <f>IFERROR(F21/E21,0)</f>
+        <v/>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -758,6 +946,16 @@
         <f>IFERROR(C22/B22,0)</f>
         <v/>
       </c>
+      <c r="E22" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="F22" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G22" s="5">
+        <f>IFERROR(F22/E22,0)</f>
+        <v/>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -775,6 +973,16 @@
         <f>IFERROR(C23/B23,0)</f>
         <v/>
       </c>
+      <c r="E23" s="4" t="n">
+        <v>11231</v>
+      </c>
+      <c r="F23" s="4" t="n">
+        <v>2239</v>
+      </c>
+      <c r="G23" s="5">
+        <f>IFERROR(F23/E23,0)</f>
+        <v/>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -792,6 +1000,16 @@
         <f>IFERROR(C24/B24,0)</f>
         <v/>
       </c>
+      <c r="E24" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="F24" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="G24" s="5">
+        <f>IFERROR(F24/E24,0)</f>
+        <v/>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -809,6 +1027,16 @@
         <f>IFERROR(C25/B25,0)</f>
         <v/>
       </c>
+      <c r="E25" s="4" t="n">
+        <v>478</v>
+      </c>
+      <c r="F25" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="G25" s="5">
+        <f>IFERROR(F25/E25,0)</f>
+        <v/>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -826,6 +1054,16 @@
         <f>IFERROR(C26/B26,0)</f>
         <v/>
       </c>
+      <c r="E26" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F26" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G26" s="5">
+        <f>IFERROR(F26/E26,0)</f>
+        <v/>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -841,6 +1079,16 @@
       </c>
       <c r="D27" s="2">
         <f>IFERROR(C27/B27,0)</f>
+        <v/>
+      </c>
+      <c r="E27" s="4" t="n">
+        <v>427747</v>
+      </c>
+      <c r="F27" s="4" t="n">
+        <v>6553</v>
+      </c>
+      <c r="G27" s="5">
+        <f>IFERROR(F27/E27,0)</f>
         <v/>
       </c>
     </row>
@@ -897,199 +1145,163 @@
     <row r="78"/>
     <row r="79"/>
     <row r="80"/>
-    <row r="81">
-      <c r="A81" s="1" t="inlineStr">
+    <row r="81"/>
+    <row r="82"/>
+    <row r="83">
+      <c r="A83" s="1" t="inlineStr">
         <is>
           <t>Gerencia</t>
         </is>
       </c>
-      <c r="B81" s="1" t="inlineStr">
+      <c r="B83" s="1" t="inlineStr">
         <is>
           <t>Cantidad alertas</t>
         </is>
       </c>
-      <c r="C81" s="1" t="inlineStr">
+      <c r="C83" s="1" t="inlineStr">
         <is>
           <t>Alertas con reproceso</t>
         </is>
       </c>
-      <c r="D81" s="1" t="inlineStr">
+      <c r="D83" s="1" t="inlineStr">
         <is>
           <t>Alertas sin reproceso</t>
         </is>
       </c>
-      <c r="E81" s="1" t="inlineStr">
+      <c r="E83" s="1" t="inlineStr">
         <is>
           <t>Calidad Gerencia</t>
         </is>
-      </c>
-    </row>
-    <row r="82">
-      <c r="A82" t="inlineStr">
-        <is>
-          <t>GCIA ESTADOS FINANCIEROS</t>
-        </is>
-      </c>
-      <c r="B82" t="n">
-        <v>170</v>
-      </c>
-      <c r="C82" t="n">
-        <v>0</v>
-      </c>
-      <c r="D82" t="n">
-        <v>170</v>
-      </c>
-      <c r="E82" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="83">
-      <c r="A83" t="inlineStr">
-        <is>
-          <t>GCIA ADMINISTRACION DEL ACTIVO</t>
-        </is>
-      </c>
-      <c r="B83" t="n">
-        <v>51</v>
-      </c>
-      <c r="C83" t="n">
-        <v>0</v>
-      </c>
-      <c r="D83" t="n">
-        <v>51</v>
-      </c>
-      <c r="E83" s="2" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>GCIA CONTABLE Y TRIBUTARIA NEQUI</t>
+          <t>GCIA ESTADOS FINANCIEROS</t>
         </is>
       </c>
       <c r="B84" t="n">
-        <v>422</v>
+        <v>170</v>
       </c>
       <c r="C84" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D84" t="n">
-        <v>417</v>
+        <v>170</v>
       </c>
       <c r="E84" s="2" t="n">
-        <v>0.01184834123222744</v>
+        <v>0</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>GCIA OPERACION MEDIOS Y ACEPTACION PAGOS</t>
+          <t>GCIA ADMINISTRACION DEL ACTIVO</t>
         </is>
       </c>
       <c r="B85" t="n">
-        <v>1544</v>
+        <v>51</v>
       </c>
       <c r="C85" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="D85" t="n">
-        <v>1529</v>
+        <v>51</v>
       </c>
       <c r="E85" s="2" t="n">
-        <v>0.009715025906735786</v>
+        <v>0</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>GCIA AUTOSERVICIOS Y EFECTIVO</t>
+          <t>GCIA CONTABLE Y TRIBUTARIA NEQUI</t>
         </is>
       </c>
       <c r="B86" t="n">
-        <v>281</v>
+        <v>422</v>
       </c>
       <c r="C86" t="n">
         <v>5</v>
       </c>
       <c r="D86" t="n">
-        <v>276</v>
+        <v>417</v>
       </c>
       <c r="E86" s="2" t="n">
-        <v>0.01779359430604988</v>
+        <v>0.01184834123222744</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>GERENCIA DE SERVICIOS DE COBRANZA Y BRP</t>
+          <t>GCIA OPERACION MEDIOS Y ACEPTACION PAGOS</t>
         </is>
       </c>
       <c r="B87" t="n">
-        <v>168</v>
+        <v>1544</v>
       </c>
       <c r="C87" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="D87" t="n">
-        <v>168</v>
+        <v>1529</v>
       </c>
       <c r="E87" s="2" t="n">
-        <v>0</v>
+        <v>0.009715025906735786</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>GCIA OPERACION DEPOSITOS PARA CLIENTES</t>
+          <t>GCIA AUTOSERVICIOS Y EFECTIVO</t>
         </is>
       </c>
       <c r="B88" t="n">
-        <v>762</v>
+        <v>281</v>
       </c>
       <c r="C88" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D88" t="n">
-        <v>762</v>
+        <v>276</v>
       </c>
       <c r="E88" s="2" t="n">
-        <v>0</v>
+        <v>0.01779359430604988</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>EVC SERVICIOS ESTRATEGICOS NEGOCIO LRU</t>
+          <t>GERENCIA DE SERVICIOS DE COBRANZA Y BRP</t>
         </is>
       </c>
       <c r="B89" t="n">
-        <v>579</v>
+        <v>168</v>
       </c>
       <c r="C89" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D89" t="n">
-        <v>576</v>
+        <v>168</v>
       </c>
       <c r="E89" s="2" t="n">
-        <v>0.005181347150259086</v>
+        <v>0</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>GCIA MONITOREO CONTROL Y CUMP TRIBUTARIO</t>
+          <t>GCIA OPERACION DEPOSITOS PARA CLIENTES</t>
         </is>
       </c>
       <c r="B90" t="n">
-        <v>7</v>
+        <v>762</v>
       </c>
       <c r="C90" t="n">
         <v>0</v>
       </c>
       <c r="D90" t="n">
-        <v>7</v>
+        <v>762</v>
       </c>
       <c r="E90" s="2" t="n">
         <v>0</v>
@@ -1098,55 +1310,55 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>GCIA OPERACIONES SEGUROS Y NUEVOS FLUJOS</t>
+          <t>EVC SERVICIOS ESTRATEGICOS NEGOCIO LRU</t>
         </is>
       </c>
       <c r="B91" t="n">
-        <v>143</v>
+        <v>579</v>
       </c>
       <c r="C91" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D91" t="n">
-        <v>143</v>
+        <v>576</v>
       </c>
       <c r="E91" s="2" t="n">
-        <v>0</v>
+        <v>0.005181347150259086</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>GERENCIA OPERACION CASH MANAGEMENT</t>
+          <t>GCIA MONITOREO CONTROL Y CUMP TRIBUTARIO</t>
         </is>
       </c>
       <c r="B92" t="n">
-        <v>186</v>
+        <v>7</v>
       </c>
       <c r="C92" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D92" t="n">
-        <v>184</v>
+        <v>7</v>
       </c>
       <c r="E92" s="2" t="n">
-        <v>0.010752688172043</v>
+        <v>0</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>GERENCIA SERVICIOS LOGISTICOS</t>
+          <t>GCIA OPERACIONES SEGUROS Y NUEVOS FLUJOS</t>
         </is>
       </c>
       <c r="B93" t="n">
-        <v>32</v>
+        <v>143</v>
       </c>
       <c r="C93" t="n">
         <v>0</v>
       </c>
       <c r="D93" t="n">
-        <v>32</v>
+        <v>143</v>
       </c>
       <c r="E93" s="2" t="n">
         <v>0</v>
@@ -1155,36 +1367,36 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>GCIA SEGURIDAD DE PERSONAS E INF FISICA</t>
+          <t>GERENCIA OPERACION CASH MANAGEMENT</t>
         </is>
       </c>
       <c r="B94" t="n">
-        <v>3</v>
+        <v>186</v>
       </c>
       <c r="C94" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D94" t="n">
-        <v>2</v>
+        <v>184</v>
       </c>
       <c r="E94" s="2" t="n">
-        <v>0.3333333333333334</v>
+        <v>0.010752688172043</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>GCIA DE CREDITO HIPOTECARIO</t>
+          <t>GERENCIA SERVICIOS LOGISTICOS</t>
         </is>
       </c>
       <c r="B95" t="n">
-        <v>4</v>
+        <v>32</v>
       </c>
       <c r="C95" t="n">
         <v>0</v>
       </c>
       <c r="D95" t="n">
-        <v>4</v>
+        <v>32</v>
       </c>
       <c r="E95" s="2" t="n">
         <v>0</v>
@@ -1193,36 +1405,36 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>GCIA GESTION INMOBILIARIA</t>
+          <t>GCIA SEGURIDAD DE PERSONAS E INF FISICA</t>
         </is>
       </c>
       <c r="B96" t="n">
-        <v>67</v>
+        <v>3</v>
       </c>
       <c r="C96" t="n">
         <v>1</v>
       </c>
       <c r="D96" t="n">
-        <v>66</v>
+        <v>2</v>
       </c>
       <c r="E96" s="2" t="n">
-        <v>0.0149253731343284</v>
+        <v>0.3333333333333334</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>GCIA ATENCION AL CLIENTE</t>
+          <t>GCIA DE CREDITO HIPOTECARIO</t>
         </is>
       </c>
       <c r="B97" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="C97" t="n">
         <v>0</v>
       </c>
       <c r="D97" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="E97" s="2" t="n">
         <v>0</v>
@@ -1231,55 +1443,55 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>GCIA DE REQUERIMIENTOS LEGALES E INSTITU</t>
+          <t>GCIA GESTION INMOBILIARIA</t>
         </is>
       </c>
       <c r="B98" t="n">
-        <v>19</v>
+        <v>67</v>
       </c>
       <c r="C98" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D98" t="n">
-        <v>19</v>
+        <v>66</v>
       </c>
       <c r="E98" s="2" t="n">
-        <v>0</v>
+        <v>0.0149253731343284</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>FOMENTO LEASING RENTA Y USO</t>
+          <t>GCIA ATENCION AL CLIENTE</t>
         </is>
       </c>
       <c r="B99" t="n">
-        <v>35</v>
+        <v>9</v>
       </c>
       <c r="C99" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D99" t="n">
-        <v>30</v>
+        <v>9</v>
       </c>
       <c r="E99" s="2" t="n">
-        <v>0.1428571428571429</v>
+        <v>0</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>GCIA ATRACCION DEL TALENTO</t>
+          <t>GCIA DE REQUERIMIENTOS LEGALES E INSTITU</t>
         </is>
       </c>
       <c r="B100" t="n">
-        <v>3</v>
+        <v>19</v>
       </c>
       <c r="C100" t="n">
         <v>0</v>
       </c>
       <c r="D100" t="n">
-        <v>3</v>
+        <v>19</v>
       </c>
       <c r="E100" s="2" t="n">
         <v>0</v>
@@ -1288,188 +1500,188 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>ADC DISEÑO Y OPERACION TELCO TI</t>
+          <t>FOMENTO LEASING RENTA Y USO</t>
         </is>
       </c>
       <c r="B101" t="n">
-        <v>1</v>
+        <v>35</v>
       </c>
       <c r="C101" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D101" t="n">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="E101" s="2" t="n">
-        <v>0</v>
+        <v>0.1428571428571429</v>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>GCIA SERV FINANCIEROS MERCADO CAPITALES</t>
+          <t>GCIA ATRACCION DEL TALENTO</t>
         </is>
       </c>
       <c r="B102" t="n">
-        <v>2594</v>
+        <v>3</v>
       </c>
       <c r="C102" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="D102" t="n">
-        <v>2588</v>
+        <v>3</v>
       </c>
       <c r="E102" s="2" t="n">
-        <v>0.002313030069390876</v>
+        <v>0</v>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>GCIA OP NEGOCIO INMOBILIARIO Y FACTORING</t>
+          <t>ADC DISEÑO Y OPERACION TELCO TI</t>
         </is>
       </c>
       <c r="B103" t="n">
-        <v>666</v>
+        <v>1</v>
       </c>
       <c r="C103" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="D103" t="n">
-        <v>659</v>
+        <v>1</v>
       </c>
       <c r="E103" s="2" t="n">
-        <v>0.01051051051051055</v>
+        <v>0</v>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>GERENCIA OPERACION DE FINANCIACION</t>
+          <t>GCIA SERV FINANCIEROS MERCADO CAPITALES</t>
         </is>
       </c>
       <c r="B104" t="n">
-        <v>874</v>
+        <v>2594</v>
       </c>
       <c r="C104" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="D104" t="n">
-        <v>874</v>
+        <v>2588</v>
       </c>
       <c r="E104" s="2" t="n">
-        <v>0</v>
+        <v>0.002313030069390876</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>GCIA SERVICIOS CONTABLES ADMINISTRATIVOS</t>
+          <t>GCIA OP NEGOCIO INMOBILIARIO Y FACTORING</t>
         </is>
       </c>
       <c r="B105" t="n">
-        <v>172</v>
+        <v>666</v>
       </c>
       <c r="C105" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="D105" t="n">
-        <v>170</v>
+        <v>659</v>
       </c>
       <c r="E105" s="2" t="n">
-        <v>0.01162790697674421</v>
+        <v>0.01051051051051055</v>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>GCIA SERVICIOS FINANCIEROS CORPORATIVOS</t>
+          <t>GERENCIA OPERACION DE FINANCIACION</t>
         </is>
       </c>
       <c r="B106" t="n">
-        <v>903</v>
+        <v>874</v>
       </c>
       <c r="C106" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D106" t="n">
-        <v>900</v>
+        <v>874</v>
       </c>
       <c r="E106" s="2" t="n">
-        <v>0.003322259136212646</v>
+        <v>0</v>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>GCIA SERVICIOS GESTION DEL FRAUDE</t>
+          <t>GCIA SERVICIOS CONTABLES ADMINISTRATIVOS</t>
         </is>
       </c>
       <c r="B107" t="n">
-        <v>87</v>
+        <v>172</v>
       </c>
       <c r="C107" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D107" t="n">
-        <v>87</v>
+        <v>170</v>
       </c>
       <c r="E107" s="2" t="n">
-        <v>0</v>
+        <v>0.01162790697674421</v>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>OPERACION Y ANALITICA ECOSISTEMAS</t>
+          <t>GCIA SERVICIOS FINANCIEROS CORPORATIVOS</t>
         </is>
       </c>
       <c r="B108" t="n">
-        <v>35</v>
+        <v>903</v>
       </c>
       <c r="C108" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D108" t="n">
-        <v>35</v>
+        <v>900</v>
       </c>
       <c r="E108" s="2" t="n">
-        <v>0</v>
+        <v>0.003322259136212646</v>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>EVC SERVICIOS PARA EL NEGOCIO SUFI</t>
+          <t>GCIA SERVICIOS GESTION DEL FRAUDE</t>
         </is>
       </c>
       <c r="B109" t="n">
-        <v>390</v>
+        <v>87</v>
       </c>
       <c r="C109" t="n">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="D109" t="n">
-        <v>376</v>
+        <v>87</v>
       </c>
       <c r="E109" s="2" t="n">
-        <v>0.03589743589743588</v>
+        <v>0</v>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>GCIA SERVICIOS DE NOMINA A EMPLEADOS</t>
+          <t>OPERACION Y ANALITICA ECOSISTEMAS</t>
         </is>
       </c>
       <c r="B110" t="n">
-        <v>99</v>
+        <v>35</v>
       </c>
       <c r="C110" t="n">
         <v>0</v>
       </c>
       <c r="D110" t="n">
-        <v>99</v>
+        <v>35</v>
       </c>
       <c r="E110" s="2" t="n">
         <v>0</v>
@@ -1478,36 +1690,36 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>GCIA DE SERV REPORTERIA LEGAL Y TRIBUT</t>
+          <t>EVC SERVICIOS PARA EL NEGOCIO SUFI</t>
         </is>
       </c>
       <c r="B111" t="n">
-        <v>36</v>
+        <v>390</v>
       </c>
       <c r="C111" t="n">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="D111" t="n">
-        <v>36</v>
+        <v>376</v>
       </c>
       <c r="E111" s="2" t="n">
-        <v>0</v>
+        <v>0.03589743589743588</v>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>GCIA DE TRANSFORMACION DE LITIGIOS</t>
+          <t>GCIA SERVICIOS DE NOMINA A EMPLEADOS</t>
         </is>
       </c>
       <c r="B112" t="n">
-        <v>16</v>
+        <v>99</v>
       </c>
       <c r="C112" t="n">
         <v>0</v>
       </c>
       <c r="D112" t="n">
-        <v>16</v>
+        <v>99</v>
       </c>
       <c r="E112" s="2" t="n">
         <v>0</v>
@@ -1516,17 +1728,17 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>ADC GESTION DE LA OPERACION</t>
+          <t>GCIA DE SERV REPORTERIA LEGAL Y TRIBUT</t>
         </is>
       </c>
       <c r="B113" t="n">
-        <v>9</v>
+        <v>36</v>
       </c>
       <c r="C113" t="n">
         <v>0</v>
       </c>
       <c r="D113" t="n">
-        <v>9</v>
+        <v>36</v>
       </c>
       <c r="E113" s="2" t="n">
         <v>0</v>
@@ -1535,17 +1747,17 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>GERENCIA OPERACIONES TALENTO Y CULTURA</t>
+          <t>GCIA DE TRANSFORMACION DE LITIGIOS</t>
         </is>
       </c>
       <c r="B114" t="n">
-        <v>2</v>
+        <v>16</v>
       </c>
       <c r="C114" t="n">
         <v>0</v>
       </c>
       <c r="D114" t="n">
-        <v>2</v>
+        <v>16</v>
       </c>
       <c r="E114" s="2" t="n">
         <v>0</v>
@@ -1554,17 +1766,17 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>LDC FC SITIO DE CONTENIDOS</t>
+          <t>ADC GESTION DE LA OPERACION</t>
         </is>
       </c>
       <c r="B115" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="C115" t="n">
         <v>0</v>
       </c>
       <c r="D115" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="E115" s="2" t="n">
         <v>0</v>
@@ -1573,17 +1785,17 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>GCIA APRENDIZAJE</t>
+          <t>GERENCIA OPERACIONES TALENTO Y CULTURA</t>
         </is>
       </c>
       <c r="B116" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C116" t="n">
         <v>0</v>
       </c>
       <c r="D116" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E116" s="2" t="n">
         <v>0</v>
@@ -1592,24 +1804,60 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
+          <t>LDC FC SITIO DE CONTENIDOS</t>
+        </is>
+      </c>
+      <c r="B117" t="n">
+        <v>1</v>
+      </c>
+      <c r="C117" t="n">
+        <v>0</v>
+      </c>
+      <c r="D117" t="n">
+        <v>1</v>
+      </c>
+      <c r="E117" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>GCIA APRENDIZAJE</t>
+        </is>
+      </c>
+      <c r="B118" t="n">
+        <v>1</v>
+      </c>
+      <c r="C118" t="n">
+        <v>0</v>
+      </c>
+      <c r="D118" t="n">
+        <v>1</v>
+      </c>
+      <c r="E118" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
           <t>Total general</t>
         </is>
       </c>
-      <c r="B117" t="n">
+      <c r="B119" t="n">
         <v>10372</v>
       </c>
-      <c r="C117" t="n">
+      <c r="C119" t="n">
         <v>69</v>
       </c>
-      <c r="D117" t="n">
+      <c r="D119" t="n">
         <v>10303</v>
       </c>
-      <c r="E117" s="2" t="n">
+      <c r="E119" s="2" t="n">
         <v>0.006652526031623585</v>
       </c>
     </row>
-    <row r="118"/>
-    <row r="119"/>
     <row r="120"/>
     <row r="121"/>
     <row r="122"/>

</xml_diff>

<commit_message>
Temporales con PARTIDAS FUERA DE POLITICA y VALOR PARTIDAS PESOS DB lista
</commit_message>
<xml_diff>
--- a/datos/salida/Indicadores_operacion_nuevo.xlsx
+++ b/datos/salida/Indicadores_operacion_nuevo.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A4:G503"/>
+  <dimension ref="A4:J303"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="4">
@@ -470,6 +470,21 @@
           <t>%</t>
         </is>
       </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>TOTAL VALOR PARTIDAS PESOS DB</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>VALOR PARTIDAS PESOS DB (Fuera de política)</t>
+        </is>
+      </c>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -497,6 +512,16 @@
         <f>IFERROR(F5/E5,0)</f>
         <v/>
       </c>
+      <c r="H5" s="4" t="n">
+        <v>8166209859</v>
+      </c>
+      <c r="I5" s="4" t="n">
+        <v>85655348</v>
+      </c>
+      <c r="J5" s="5">
+        <f>IFERROR(I5/H5,0)</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -524,6 +549,16 @@
         <f>IFERROR(F6/E6,0)</f>
         <v/>
       </c>
+      <c r="H6" s="4" t="n">
+        <v>169629603</v>
+      </c>
+      <c r="I6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J6" s="5">
+        <f>IFERROR(I6/H6,0)</f>
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -551,6 +586,16 @@
         <f>IFERROR(F7/E7,0)</f>
         <v/>
       </c>
+      <c r="H7" s="4" t="n">
+        <v>19530072</v>
+      </c>
+      <c r="I7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J7" s="5">
+        <f>IFERROR(I7/H7,0)</f>
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -578,6 +623,16 @@
         <f>IFERROR(F8/E8,0)</f>
         <v/>
       </c>
+      <c r="H8" s="4" t="n">
+        <v>46528879540</v>
+      </c>
+      <c r="I8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J8" s="5">
+        <f>IFERROR(I8/H8,0)</f>
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -605,6 +660,16 @@
         <f>IFERROR(F9/E9,0)</f>
         <v/>
       </c>
+      <c r="H9" s="4" t="n">
+        <v>476282522355</v>
+      </c>
+      <c r="I9" s="4" t="n">
+        <v>131262339</v>
+      </c>
+      <c r="J9" s="5">
+        <f>IFERROR(I9/H9,0)</f>
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -632,6 +697,16 @@
         <f>IFERROR(F10/E10,0)</f>
         <v/>
       </c>
+      <c r="H10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J10" s="5">
+        <f>IFERROR(I10/H10,0)</f>
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -659,6 +734,16 @@
         <f>IFERROR(F11/E11,0)</f>
         <v/>
       </c>
+      <c r="H11" s="4" t="n">
+        <v>879354000</v>
+      </c>
+      <c r="I11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J11" s="5">
+        <f>IFERROR(I11/H11,0)</f>
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -686,6 +771,16 @@
         <f>IFERROR(F12/E12,0)</f>
         <v/>
       </c>
+      <c r="H12" s="4" t="n">
+        <v>49387269</v>
+      </c>
+      <c r="I12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J12" s="5">
+        <f>IFERROR(I12/H12,0)</f>
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -713,6 +808,16 @@
         <f>IFERROR(F13/E13,0)</f>
         <v/>
       </c>
+      <c r="H13" s="4" t="n">
+        <v>2067009200</v>
+      </c>
+      <c r="I13" s="4" t="n">
+        <v>1385225</v>
+      </c>
+      <c r="J13" s="5">
+        <f>IFERROR(I13/H13,0)</f>
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -740,6 +845,16 @@
         <f>IFERROR(F14/E14,0)</f>
         <v/>
       </c>
+      <c r="H14" s="4" t="n">
+        <v>4611807738</v>
+      </c>
+      <c r="I14" s="4" t="n">
+        <v>100379182</v>
+      </c>
+      <c r="J14" s="5">
+        <f>IFERROR(I14/H14,0)</f>
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -767,6 +882,16 @@
         <f>IFERROR(F15/E15,0)</f>
         <v/>
       </c>
+      <c r="H15" s="4" t="n">
+        <v>434893556327</v>
+      </c>
+      <c r="I15" s="4" t="n">
+        <v>2043654363</v>
+      </c>
+      <c r="J15" s="5">
+        <f>IFERROR(I15/H15,0)</f>
+        <v/>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -794,6 +919,16 @@
         <f>IFERROR(F16/E16,0)</f>
         <v/>
       </c>
+      <c r="H16" s="4" t="n">
+        <v>1025947950</v>
+      </c>
+      <c r="I16" s="4" t="n">
+        <v>1025947950</v>
+      </c>
+      <c r="J16" s="5">
+        <f>IFERROR(I16/H16,0)</f>
+        <v/>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -821,6 +956,16 @@
         <f>IFERROR(F17/E17,0)</f>
         <v/>
       </c>
+      <c r="H17" s="4" t="n">
+        <v>53569914</v>
+      </c>
+      <c r="I17" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J17" s="5">
+        <f>IFERROR(I17/H17,0)</f>
+        <v/>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -848,6 +993,16 @@
         <f>IFERROR(F18/E18,0)</f>
         <v/>
       </c>
+      <c r="H18" s="4" t="n">
+        <v>1735186694</v>
+      </c>
+      <c r="I18" s="4" t="n">
+        <v>119938287</v>
+      </c>
+      <c r="J18" s="5">
+        <f>IFERROR(I18/H18,0)</f>
+        <v/>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -875,6 +1030,16 @@
         <f>IFERROR(F19/E19,0)</f>
         <v/>
       </c>
+      <c r="H19" s="4" t="n">
+        <v>272959617</v>
+      </c>
+      <c r="I19" s="4" t="n">
+        <v>215364473</v>
+      </c>
+      <c r="J19" s="5">
+        <f>IFERROR(I19/H19,0)</f>
+        <v/>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -902,6 +1067,16 @@
         <f>IFERROR(F20/E20,0)</f>
         <v/>
       </c>
+      <c r="H20" s="4" t="n">
+        <v>100730000</v>
+      </c>
+      <c r="I20" s="4" t="n">
+        <v>100730000</v>
+      </c>
+      <c r="J20" s="5">
+        <f>IFERROR(I20/H20,0)</f>
+        <v/>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -929,6 +1104,16 @@
         <f>IFERROR(F21/E21,0)</f>
         <v/>
       </c>
+      <c r="H21" s="4" t="n">
+        <v>10453116046</v>
+      </c>
+      <c r="I21" s="4" t="n">
+        <v>757215</v>
+      </c>
+      <c r="J21" s="5">
+        <f>IFERROR(I21/H21,0)</f>
+        <v/>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -956,6 +1141,16 @@
         <f>IFERROR(F22/E22,0)</f>
         <v/>
       </c>
+      <c r="H22" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I22" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J22" s="5">
+        <f>IFERROR(I22/H22,0)</f>
+        <v/>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -983,6 +1178,16 @@
         <f>IFERROR(F23/E23,0)</f>
         <v/>
       </c>
+      <c r="H23" s="4" t="n">
+        <v>7418616076</v>
+      </c>
+      <c r="I23" s="4" t="n">
+        <v>3307034014</v>
+      </c>
+      <c r="J23" s="5">
+        <f>IFERROR(I23/H23,0)</f>
+        <v/>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1010,6 +1215,16 @@
         <f>IFERROR(F24/E24,0)</f>
         <v/>
       </c>
+      <c r="H24" s="4" t="n">
+        <v>125581419</v>
+      </c>
+      <c r="I24" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J24" s="5">
+        <f>IFERROR(I24/H24,0)</f>
+        <v/>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1037,6 +1252,16 @@
         <f>IFERROR(F25/E25,0)</f>
         <v/>
       </c>
+      <c r="H25" s="4" t="n">
+        <v>600000</v>
+      </c>
+      <c r="I25" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J25" s="5">
+        <f>IFERROR(I25/H25,0)</f>
+        <v/>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1064,6 +1289,16 @@
         <f>IFERROR(F26/E26,0)</f>
         <v/>
       </c>
+      <c r="H26" s="4" t="n">
+        <v>376589540</v>
+      </c>
+      <c r="I26" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J26" s="5">
+        <f>IFERROR(I26/H26,0)</f>
+        <v/>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1089,6 +1324,16 @@
       </c>
       <c r="G27" s="5">
         <f>IFERROR(F27/E27,0)</f>
+        <v/>
+      </c>
+      <c r="H27" s="4" t="n">
+        <v>995230783229</v>
+      </c>
+      <c r="I27" s="4" t="n">
+        <v>7132108399</v>
+      </c>
+      <c r="J27" s="5">
+        <f>IFERROR(I27/H27,0)</f>
         <v/>
       </c>
     </row>
@@ -2991,206 +3236,6 @@
     <row r="301"/>
     <row r="302"/>
     <row r="303"/>
-    <row r="304"/>
-    <row r="305"/>
-    <row r="306"/>
-    <row r="307"/>
-    <row r="308"/>
-    <row r="309"/>
-    <row r="310"/>
-    <row r="311"/>
-    <row r="312"/>
-    <row r="313"/>
-    <row r="314"/>
-    <row r="315"/>
-    <row r="316"/>
-    <row r="317"/>
-    <row r="318"/>
-    <row r="319"/>
-    <row r="320"/>
-    <row r="321"/>
-    <row r="322"/>
-    <row r="323"/>
-    <row r="324"/>
-    <row r="325"/>
-    <row r="326"/>
-    <row r="327"/>
-    <row r="328"/>
-    <row r="329"/>
-    <row r="330"/>
-    <row r="331"/>
-    <row r="332"/>
-    <row r="333"/>
-    <row r="334"/>
-    <row r="335"/>
-    <row r="336"/>
-    <row r="337"/>
-    <row r="338"/>
-    <row r="339"/>
-    <row r="340"/>
-    <row r="341"/>
-    <row r="342"/>
-    <row r="343"/>
-    <row r="344"/>
-    <row r="345"/>
-    <row r="346"/>
-    <row r="347"/>
-    <row r="348"/>
-    <row r="349"/>
-    <row r="350"/>
-    <row r="351"/>
-    <row r="352"/>
-    <row r="353"/>
-    <row r="354"/>
-    <row r="355"/>
-    <row r="356"/>
-    <row r="357"/>
-    <row r="358"/>
-    <row r="359"/>
-    <row r="360"/>
-    <row r="361"/>
-    <row r="362"/>
-    <row r="363"/>
-    <row r="364"/>
-    <row r="365"/>
-    <row r="366"/>
-    <row r="367"/>
-    <row r="368"/>
-    <row r="369"/>
-    <row r="370"/>
-    <row r="371"/>
-    <row r="372"/>
-    <row r="373"/>
-    <row r="374"/>
-    <row r="375"/>
-    <row r="376"/>
-    <row r="377"/>
-    <row r="378"/>
-    <row r="379"/>
-    <row r="380"/>
-    <row r="381"/>
-    <row r="382"/>
-    <row r="383"/>
-    <row r="384"/>
-    <row r="385"/>
-    <row r="386"/>
-    <row r="387"/>
-    <row r="388"/>
-    <row r="389"/>
-    <row r="390"/>
-    <row r="391"/>
-    <row r="392"/>
-    <row r="393"/>
-    <row r="394"/>
-    <row r="395"/>
-    <row r="396"/>
-    <row r="397"/>
-    <row r="398"/>
-    <row r="399"/>
-    <row r="400"/>
-    <row r="401"/>
-    <row r="402"/>
-    <row r="403"/>
-    <row r="404"/>
-    <row r="405"/>
-    <row r="406"/>
-    <row r="407"/>
-    <row r="408"/>
-    <row r="409"/>
-    <row r="410"/>
-    <row r="411"/>
-    <row r="412"/>
-    <row r="413"/>
-    <row r="414"/>
-    <row r="415"/>
-    <row r="416"/>
-    <row r="417"/>
-    <row r="418"/>
-    <row r="419"/>
-    <row r="420"/>
-    <row r="421"/>
-    <row r="422"/>
-    <row r="423"/>
-    <row r="424"/>
-    <row r="425"/>
-    <row r="426"/>
-    <row r="427"/>
-    <row r="428"/>
-    <row r="429"/>
-    <row r="430"/>
-    <row r="431"/>
-    <row r="432"/>
-    <row r="433"/>
-    <row r="434"/>
-    <row r="435"/>
-    <row r="436"/>
-    <row r="437"/>
-    <row r="438"/>
-    <row r="439"/>
-    <row r="440"/>
-    <row r="441"/>
-    <row r="442"/>
-    <row r="443"/>
-    <row r="444"/>
-    <row r="445"/>
-    <row r="446"/>
-    <row r="447"/>
-    <row r="448"/>
-    <row r="449"/>
-    <row r="450"/>
-    <row r="451"/>
-    <row r="452"/>
-    <row r="453"/>
-    <row r="454"/>
-    <row r="455"/>
-    <row r="456"/>
-    <row r="457"/>
-    <row r="458"/>
-    <row r="459"/>
-    <row r="460"/>
-    <row r="461"/>
-    <row r="462"/>
-    <row r="463"/>
-    <row r="464"/>
-    <row r="465"/>
-    <row r="466"/>
-    <row r="467"/>
-    <row r="468"/>
-    <row r="469"/>
-    <row r="470"/>
-    <row r="471"/>
-    <row r="472"/>
-    <row r="473"/>
-    <row r="474"/>
-    <row r="475"/>
-    <row r="476"/>
-    <row r="477"/>
-    <row r="478"/>
-    <row r="479"/>
-    <row r="480"/>
-    <row r="481"/>
-    <row r="482"/>
-    <row r="483"/>
-    <row r="484"/>
-    <row r="485"/>
-    <row r="486"/>
-    <row r="487"/>
-    <row r="488"/>
-    <row r="489"/>
-    <row r="490"/>
-    <row r="491"/>
-    <row r="492"/>
-    <row r="493"/>
-    <row r="494"/>
-    <row r="495"/>
-    <row r="496"/>
-    <row r="497"/>
-    <row r="498"/>
-    <row r="499"/>
-    <row r="500"/>
-    <row r="501"/>
-    <row r="502"/>
-    <row r="503"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
TD SABANA DB y CR completos; exporte a Indicadores (A4/E4/H4/K4). Pendiente optimización y ajuste de sobrescritura
</commit_message>
<xml_diff>
--- a/datos/salida/Indicadores_operacion_nuevo.xlsx
+++ b/datos/salida/Indicadores_operacion_nuevo.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A4:J303"/>
+  <dimension ref="A4:M303"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="4">
@@ -485,6 +485,21 @@
           <t>%</t>
         </is>
       </c>
+      <c r="K4" s="3" t="inlineStr">
+        <is>
+          <t>TOTAL VALOR PARTIDAS PESOS CR</t>
+        </is>
+      </c>
+      <c r="L4" s="3" t="inlineStr">
+        <is>
+          <t>VALOR PARTIDAS PESOS CR (Fuera de política)</t>
+        </is>
+      </c>
+      <c r="M4" s="3" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -522,6 +537,16 @@
         <f>IFERROR(I5/H5,0)</f>
         <v/>
       </c>
+      <c r="K5" s="4" t="n">
+        <v>-23495941756</v>
+      </c>
+      <c r="L5" s="4" t="n">
+        <v>-6355911</v>
+      </c>
+      <c r="M5" s="5">
+        <f>IFERROR(L5/K5,0)</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -559,6 +584,16 @@
         <f>IFERROR(I6/H6,0)</f>
         <v/>
       </c>
+      <c r="K6" s="4" t="n">
+        <v>-12415536733</v>
+      </c>
+      <c r="L6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M6" s="5">
+        <f>IFERROR(L6/K6,0)</f>
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -596,6 +631,16 @@
         <f>IFERROR(I7/H7,0)</f>
         <v/>
       </c>
+      <c r="K7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M7" s="5">
+        <f>IFERROR(L7/K7,0)</f>
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -633,6 +678,16 @@
         <f>IFERROR(I8/H8,0)</f>
         <v/>
       </c>
+      <c r="K8" s="4" t="n">
+        <v>-74870028</v>
+      </c>
+      <c r="L8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M8" s="5">
+        <f>IFERROR(L8/K8,0)</f>
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -670,6 +725,16 @@
         <f>IFERROR(I9/H9,0)</f>
         <v/>
       </c>
+      <c r="K9" s="4" t="n">
+        <v>-732062166155</v>
+      </c>
+      <c r="L9" s="4" t="n">
+        <v>-16150422</v>
+      </c>
+      <c r="M9" s="5">
+        <f>IFERROR(L9/K9,0)</f>
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -707,6 +772,16 @@
         <f>IFERROR(I10/H10,0)</f>
         <v/>
       </c>
+      <c r="K10" s="4" t="n">
+        <v>-1080629105</v>
+      </c>
+      <c r="L10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M10" s="5">
+        <f>IFERROR(L10/K10,0)</f>
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -744,6 +819,16 @@
         <f>IFERROR(I11/H11,0)</f>
         <v/>
       </c>
+      <c r="K11" s="4" t="n">
+        <v>-45857000</v>
+      </c>
+      <c r="L11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M11" s="5">
+        <f>IFERROR(L11/K11,0)</f>
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -781,6 +866,16 @@
         <f>IFERROR(I12/H12,0)</f>
         <v/>
       </c>
+      <c r="K12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M12" s="5">
+        <f>IFERROR(L12/K12,0)</f>
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -818,6 +913,16 @@
         <f>IFERROR(I13/H13,0)</f>
         <v/>
       </c>
+      <c r="K13" s="4" t="n">
+        <v>-111380482349</v>
+      </c>
+      <c r="L13" s="4" t="n">
+        <v>-3638405740</v>
+      </c>
+      <c r="M13" s="5">
+        <f>IFERROR(L13/K13,0)</f>
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -855,6 +960,16 @@
         <f>IFERROR(I14/H14,0)</f>
         <v/>
       </c>
+      <c r="K14" s="4" t="n">
+        <v>-17537201935</v>
+      </c>
+      <c r="L14" s="4" t="n">
+        <v>-137745388</v>
+      </c>
+      <c r="M14" s="5">
+        <f>IFERROR(L14/K14,0)</f>
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -892,6 +1007,16 @@
         <f>IFERROR(I15/H15,0)</f>
         <v/>
       </c>
+      <c r="K15" s="4" t="n">
+        <v>-1106195942843</v>
+      </c>
+      <c r="L15" s="4" t="n">
+        <v>-318710188</v>
+      </c>
+      <c r="M15" s="5">
+        <f>IFERROR(L15/K15,0)</f>
+        <v/>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -929,6 +1054,16 @@
         <f>IFERROR(I16/H16,0)</f>
         <v/>
       </c>
+      <c r="K16" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L16" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M16" s="5">
+        <f>IFERROR(L16/K16,0)</f>
+        <v/>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -966,6 +1101,16 @@
         <f>IFERROR(I17/H17,0)</f>
         <v/>
       </c>
+      <c r="K17" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L17" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M17" s="5">
+        <f>IFERROR(L17/K17,0)</f>
+        <v/>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1003,6 +1148,16 @@
         <f>IFERROR(I18/H18,0)</f>
         <v/>
       </c>
+      <c r="K18" s="4" t="n">
+        <v>-13080139230</v>
+      </c>
+      <c r="L18" s="4" t="n">
+        <v>-5635620000</v>
+      </c>
+      <c r="M18" s="5">
+        <f>IFERROR(L18/K18,0)</f>
+        <v/>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1040,6 +1195,16 @@
         <f>IFERROR(I19/H19,0)</f>
         <v/>
       </c>
+      <c r="K19" s="4" t="n">
+        <v>-103721808</v>
+      </c>
+      <c r="L19" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M19" s="5">
+        <f>IFERROR(L19/K19,0)</f>
+        <v/>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1077,6 +1242,16 @@
         <f>IFERROR(I20/H20,0)</f>
         <v/>
       </c>
+      <c r="K20" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L20" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M20" s="5">
+        <f>IFERROR(L20/K20,0)</f>
+        <v/>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1114,6 +1289,16 @@
         <f>IFERROR(I21/H21,0)</f>
         <v/>
       </c>
+      <c r="K21" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L21" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M21" s="5">
+        <f>IFERROR(L21/K21,0)</f>
+        <v/>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1151,6 +1336,16 @@
         <f>IFERROR(I22/H22,0)</f>
         <v/>
       </c>
+      <c r="K22" s="4" t="n">
+        <v>-122292274</v>
+      </c>
+      <c r="L22" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M22" s="5">
+        <f>IFERROR(L22/K22,0)</f>
+        <v/>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1188,6 +1383,16 @@
         <f>IFERROR(I23/H23,0)</f>
         <v/>
       </c>
+      <c r="K23" s="4" t="n">
+        <v>-8645359507</v>
+      </c>
+      <c r="L23" s="4" t="n">
+        <v>-2517783400</v>
+      </c>
+      <c r="M23" s="5">
+        <f>IFERROR(L23/K23,0)</f>
+        <v/>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1225,6 +1430,16 @@
         <f>IFERROR(I24/H24,0)</f>
         <v/>
       </c>
+      <c r="K24" s="4" t="n">
+        <v>-460064217187</v>
+      </c>
+      <c r="L24" s="4" t="n">
+        <v>-10363107</v>
+      </c>
+      <c r="M24" s="5">
+        <f>IFERROR(L24/K24,0)</f>
+        <v/>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1262,6 +1477,16 @@
         <f>IFERROR(I25/H25,0)</f>
         <v/>
       </c>
+      <c r="K25" s="4" t="n">
+        <v>-9791219529</v>
+      </c>
+      <c r="L25" s="4" t="n">
+        <v>-6810293</v>
+      </c>
+      <c r="M25" s="5">
+        <f>IFERROR(L25/K25,0)</f>
+        <v/>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1299,6 +1524,16 @@
         <f>IFERROR(I26/H26,0)</f>
         <v/>
       </c>
+      <c r="K26" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L26" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M26" s="5">
+        <f>IFERROR(L26/K26,0)</f>
+        <v/>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1336,53 +1571,799 @@
         <f>IFERROR(I27/H27,0)</f>
         <v/>
       </c>
-    </row>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
-    <row r="32"/>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
-    <row r="40"/>
-    <row r="41"/>
-    <row r="42"/>
-    <row r="43"/>
-    <row r="44"/>
-    <row r="45"/>
-    <row r="46"/>
-    <row r="47"/>
-    <row r="48"/>
-    <row r="49"/>
-    <row r="50"/>
-    <row r="51"/>
-    <row r="52"/>
-    <row r="53"/>
-    <row r="54"/>
-    <row r="55"/>
-    <row r="56"/>
-    <row r="57"/>
-    <row r="58"/>
-    <row r="59"/>
-    <row r="60"/>
-    <row r="61"/>
-    <row r="62"/>
-    <row r="63"/>
-    <row r="64"/>
-    <row r="65"/>
-    <row r="66"/>
-    <row r="67"/>
-    <row r="68"/>
-    <row r="69"/>
-    <row r="70"/>
-    <row r="71"/>
-    <row r="72"/>
-    <row r="73"/>
+      <c r="K27" s="4" t="n">
+        <v>-2496095577444</v>
+      </c>
+      <c r="L27" s="4" t="n">
+        <v>-12287944452</v>
+      </c>
+      <c r="M27" s="5">
+        <f>IFERROR(L27/K27,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="E28" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F28" s="4" t="n">
+        <v>8166209859</v>
+      </c>
+      <c r="G28" s="5">
+        <f>IFERROR(F28/E28,0)</f>
+        <v/>
+      </c>
+      <c r="H28" s="4" t="n">
+        <v>-23495941756</v>
+      </c>
+      <c r="I28" s="4" t="n">
+        <v>-6355911</v>
+      </c>
+      <c r="J28" s="5">
+        <f>IFERROR(I28/H28,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="E29" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F29" s="4" t="n">
+        <v>169629603</v>
+      </c>
+      <c r="G29" s="5">
+        <f>IFERROR(F29/E29,0)</f>
+        <v/>
+      </c>
+      <c r="H29" s="4" t="n">
+        <v>-12415536733</v>
+      </c>
+      <c r="I29" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J29" s="5">
+        <f>IFERROR(I29/H29,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="E30" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F30" s="4" t="n">
+        <v>19530072</v>
+      </c>
+      <c r="G30" s="5">
+        <f>IFERROR(F30/E30,0)</f>
+        <v/>
+      </c>
+      <c r="H30" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I30" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J30" s="5">
+        <f>IFERROR(I30/H30,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="E31" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F31" s="4" t="n">
+        <v>46528879540</v>
+      </c>
+      <c r="G31" s="5">
+        <f>IFERROR(F31/E31,0)</f>
+        <v/>
+      </c>
+      <c r="H31" s="4" t="n">
+        <v>-74870028</v>
+      </c>
+      <c r="I31" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J31" s="5">
+        <f>IFERROR(I31/H31,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="E32" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F32" s="4" t="n">
+        <v>476282522355</v>
+      </c>
+      <c r="G32" s="5">
+        <f>IFERROR(F32/E32,0)</f>
+        <v/>
+      </c>
+      <c r="H32" s="4" t="n">
+        <v>-732062166155</v>
+      </c>
+      <c r="I32" s="4" t="n">
+        <v>-16150422</v>
+      </c>
+      <c r="J32" s="5">
+        <f>IFERROR(I32/H32,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="E33" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F33" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G33" s="5">
+        <f>IFERROR(F33/E33,0)</f>
+        <v/>
+      </c>
+      <c r="H33" s="4" t="n">
+        <v>-1080629105</v>
+      </c>
+      <c r="I33" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J33" s="5">
+        <f>IFERROR(I33/H33,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="E34" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F34" s="4" t="n">
+        <v>879354000</v>
+      </c>
+      <c r="G34" s="5">
+        <f>IFERROR(F34/E34,0)</f>
+        <v/>
+      </c>
+      <c r="H34" s="4" t="n">
+        <v>-45857000</v>
+      </c>
+      <c r="I34" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J34" s="5">
+        <f>IFERROR(I34/H34,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="E35" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F35" s="4" t="n">
+        <v>49387269</v>
+      </c>
+      <c r="G35" s="5">
+        <f>IFERROR(F35/E35,0)</f>
+        <v/>
+      </c>
+      <c r="H35" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I35" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J35" s="5">
+        <f>IFERROR(I35/H35,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="E36" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F36" s="4" t="n">
+        <v>2067009200</v>
+      </c>
+      <c r="G36" s="5">
+        <f>IFERROR(F36/E36,0)</f>
+        <v/>
+      </c>
+      <c r="H36" s="4" t="n">
+        <v>-111380482349</v>
+      </c>
+      <c r="I36" s="4" t="n">
+        <v>-3638405740</v>
+      </c>
+      <c r="J36" s="5">
+        <f>IFERROR(I36/H36,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="E37" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F37" s="4" t="n">
+        <v>4611807738</v>
+      </c>
+      <c r="G37" s="5">
+        <f>IFERROR(F37/E37,0)</f>
+        <v/>
+      </c>
+      <c r="H37" s="4" t="n">
+        <v>-17537201935</v>
+      </c>
+      <c r="I37" s="4" t="n">
+        <v>-137745388</v>
+      </c>
+      <c r="J37" s="5">
+        <f>IFERROR(I37/H37,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="E38" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F38" s="4" t="n">
+        <v>434893556327</v>
+      </c>
+      <c r="G38" s="5">
+        <f>IFERROR(F38/E38,0)</f>
+        <v/>
+      </c>
+      <c r="H38" s="4" t="n">
+        <v>-1106195942843</v>
+      </c>
+      <c r="I38" s="4" t="n">
+        <v>-318710188</v>
+      </c>
+      <c r="J38" s="5">
+        <f>IFERROR(I38/H38,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="E39" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F39" s="4" t="n">
+        <v>1025947950</v>
+      </c>
+      <c r="G39" s="5">
+        <f>IFERROR(F39/E39,0)</f>
+        <v/>
+      </c>
+      <c r="H39" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I39" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J39" s="5">
+        <f>IFERROR(I39/H39,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="E40" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F40" s="4" t="n">
+        <v>53569914</v>
+      </c>
+      <c r="G40" s="5">
+        <f>IFERROR(F40/E40,0)</f>
+        <v/>
+      </c>
+      <c r="H40" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I40" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J40" s="5">
+        <f>IFERROR(I40/H40,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="E41" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F41" s="4" t="n">
+        <v>1735186694</v>
+      </c>
+      <c r="G41" s="5">
+        <f>IFERROR(F41/E41,0)</f>
+        <v/>
+      </c>
+      <c r="H41" s="4" t="n">
+        <v>-13080139230</v>
+      </c>
+      <c r="I41" s="4" t="n">
+        <v>-5635620000</v>
+      </c>
+      <c r="J41" s="5">
+        <f>IFERROR(I41/H41,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="E42" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F42" s="4" t="n">
+        <v>272959617</v>
+      </c>
+      <c r="G42" s="5">
+        <f>IFERROR(F42/E42,0)</f>
+        <v/>
+      </c>
+      <c r="H42" s="4" t="n">
+        <v>-103721808</v>
+      </c>
+      <c r="I42" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J42" s="5">
+        <f>IFERROR(I42/H42,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="E43" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F43" s="4" t="n">
+        <v>100730000</v>
+      </c>
+      <c r="G43" s="5">
+        <f>IFERROR(F43/E43,0)</f>
+        <v/>
+      </c>
+      <c r="H43" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I43" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J43" s="5">
+        <f>IFERROR(I43/H43,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="E44" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F44" s="4" t="n">
+        <v>10453116046</v>
+      </c>
+      <c r="G44" s="5">
+        <f>IFERROR(F44/E44,0)</f>
+        <v/>
+      </c>
+      <c r="H44" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I44" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J44" s="5">
+        <f>IFERROR(I44/H44,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="E45" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F45" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G45" s="5">
+        <f>IFERROR(F45/E45,0)</f>
+        <v/>
+      </c>
+      <c r="H45" s="4" t="n">
+        <v>-122292274</v>
+      </c>
+      <c r="I45" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J45" s="5">
+        <f>IFERROR(I45/H45,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="E46" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F46" s="4" t="n">
+        <v>7418616076</v>
+      </c>
+      <c r="G46" s="5">
+        <f>IFERROR(F46/E46,0)</f>
+        <v/>
+      </c>
+      <c r="H46" s="4" t="n">
+        <v>-8645359507</v>
+      </c>
+      <c r="I46" s="4" t="n">
+        <v>-2517783400</v>
+      </c>
+      <c r="J46" s="5">
+        <f>IFERROR(I46/H46,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47">
+      <c r="E47" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F47" s="4" t="n">
+        <v>125581419</v>
+      </c>
+      <c r="G47" s="5">
+        <f>IFERROR(F47/E47,0)</f>
+        <v/>
+      </c>
+      <c r="H47" s="4" t="n">
+        <v>-460064217187</v>
+      </c>
+      <c r="I47" s="4" t="n">
+        <v>-10363107</v>
+      </c>
+      <c r="J47" s="5">
+        <f>IFERROR(I47/H47,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="48">
+      <c r="E48" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F48" s="4" t="n">
+        <v>600000</v>
+      </c>
+      <c r="G48" s="5">
+        <f>IFERROR(F48/E48,0)</f>
+        <v/>
+      </c>
+      <c r="H48" s="4" t="n">
+        <v>-9791219529</v>
+      </c>
+      <c r="I48" s="4" t="n">
+        <v>-6810293</v>
+      </c>
+      <c r="J48" s="5">
+        <f>IFERROR(I48/H48,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49">
+      <c r="E49" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F49" s="4" t="n">
+        <v>376589540</v>
+      </c>
+      <c r="G49" s="5">
+        <f>IFERROR(F49/E49,0)</f>
+        <v/>
+      </c>
+      <c r="H49" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I49" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J49" s="5">
+        <f>IFERROR(I49/H49,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50">
+      <c r="E50" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F50" s="4" t="n">
+        <v>995230783229</v>
+      </c>
+      <c r="G50" s="5">
+        <f>IFERROR(F50/E50,0)</f>
+        <v/>
+      </c>
+      <c r="H50" s="4" t="n">
+        <v>-2496095577444</v>
+      </c>
+      <c r="I50" s="4" t="n">
+        <v>-12287944452</v>
+      </c>
+      <c r="J50" s="5">
+        <f>IFERROR(I50/H50,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51">
+      <c r="E51" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F51" s="4" t="n">
+        <v>-23495941756</v>
+      </c>
+      <c r="G51" s="5">
+        <f>IFERROR(F51/E51,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="52">
+      <c r="E52" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F52" s="4" t="n">
+        <v>-12415536733</v>
+      </c>
+      <c r="G52" s="5">
+        <f>IFERROR(F52/E52,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="53">
+      <c r="E53" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F53" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G53" s="5">
+        <f>IFERROR(F53/E53,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="54">
+      <c r="E54" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F54" s="4" t="n">
+        <v>-74870028</v>
+      </c>
+      <c r="G54" s="5">
+        <f>IFERROR(F54/E54,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55">
+      <c r="E55" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F55" s="4" t="n">
+        <v>-732062166155</v>
+      </c>
+      <c r="G55" s="5">
+        <f>IFERROR(F55/E55,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="56">
+      <c r="E56" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F56" s="4" t="n">
+        <v>-1080629105</v>
+      </c>
+      <c r="G56" s="5">
+        <f>IFERROR(F56/E56,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="57">
+      <c r="E57" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F57" s="4" t="n">
+        <v>-45857000</v>
+      </c>
+      <c r="G57" s="5">
+        <f>IFERROR(F57/E57,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="58">
+      <c r="E58" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F58" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G58" s="5">
+        <f>IFERROR(F58/E58,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="59">
+      <c r="E59" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F59" s="4" t="n">
+        <v>-111380482349</v>
+      </c>
+      <c r="G59" s="5">
+        <f>IFERROR(F59/E59,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="60">
+      <c r="E60" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F60" s="4" t="n">
+        <v>-17537201935</v>
+      </c>
+      <c r="G60" s="5">
+        <f>IFERROR(F60/E60,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="61">
+      <c r="E61" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F61" s="4" t="n">
+        <v>-1106195942843</v>
+      </c>
+      <c r="G61" s="5">
+        <f>IFERROR(F61/E61,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="62">
+      <c r="E62" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F62" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G62" s="5">
+        <f>IFERROR(F62/E62,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="63">
+      <c r="E63" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F63" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G63" s="5">
+        <f>IFERROR(F63/E63,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="64">
+      <c r="E64" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F64" s="4" t="n">
+        <v>-13080139230</v>
+      </c>
+      <c r="G64" s="5">
+        <f>IFERROR(F64/E64,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="65">
+      <c r="E65" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F65" s="4" t="n">
+        <v>-103721808</v>
+      </c>
+      <c r="G65" s="5">
+        <f>IFERROR(F65/E65,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="66">
+      <c r="E66" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F66" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G66" s="5">
+        <f>IFERROR(F66/E66,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="67">
+      <c r="E67" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F67" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G67" s="5">
+        <f>IFERROR(F67/E67,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="68">
+      <c r="E68" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F68" s="4" t="n">
+        <v>-122292274</v>
+      </c>
+      <c r="G68" s="5">
+        <f>IFERROR(F68/E68,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="69">
+      <c r="E69" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F69" s="4" t="n">
+        <v>-8645359507</v>
+      </c>
+      <c r="G69" s="5">
+        <f>IFERROR(F69/E69,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="70">
+      <c r="E70" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F70" s="4" t="n">
+        <v>-460064217187</v>
+      </c>
+      <c r="G70" s="5">
+        <f>IFERROR(F70/E70,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="71">
+      <c r="E71" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F71" s="4" t="n">
+        <v>-9791219529</v>
+      </c>
+      <c r="G71" s="5">
+        <f>IFERROR(F71/E71,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="72">
+      <c r="E72" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F72" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G72" s="5">
+        <f>IFERROR(F72/E72,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="73">
+      <c r="E73" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F73" s="4" t="n">
+        <v>-2496095577444</v>
+      </c>
+      <c r="G73" s="5">
+        <f>IFERROR(F73/E73,0)</f>
+        <v/>
+      </c>
+    </row>
     <row r="74"/>
     <row r="75"/>
     <row r="76"/>

</xml_diff>